<commit_message>
updated to remove prev question
</commit_message>
<xml_diff>
--- a/active_practice_tests.xlsx
+++ b/active_practice_tests.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2101" uniqueCount="1375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2094" uniqueCount="1371">
   <si>
     <t xml:space="preserve">Number</t>
   </si>
@@ -5627,21 +5627,6 @@
     <t xml:space="preserve">A set comprehension</t>
   </si>
   <si>
-    <t xml:space="preserve">What is the output of the code in the previous question?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0, 1, 2]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0, 2, 4]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[2, 4, 6]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[1, 2, 4]</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -6360,6 +6345,9 @@
   </si>
   <si>
     <t xml:space="preserve">[0, 1, 2, 3]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0, 1, 2]</t>
   </si>
   <si>
     <t xml:space="preserve">(0, 1, 2)</t>
@@ -8394,8 +8382,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:J300"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="60.94"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -16208,11 +16199,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="245" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="245" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="2" t="n">
-        <v>244</v>
-      </c>
-      <c r="B245" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B245" s="4" t="s">
         <v>1105</v>
       </c>
       <c r="C245" s="3" t="s">
@@ -16227,8 +16218,8 @@
       <c r="F245" s="3" t="s">
         <v>1109</v>
       </c>
-      <c r="G245" s="2" t="n">
-        <v>2</v>
+      <c r="G245" s="2" t="s">
+        <v>134</v>
       </c>
       <c r="H245" s="2" t="s">
         <v>110</v>
@@ -16240,11 +16231,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="246" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="2" t="n">
-        <v>245</v>
-      </c>
-      <c r="B246" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="B246" s="2" t="s">
         <v>1110</v>
       </c>
       <c r="C246" s="3" t="s">
@@ -16259,11 +16250,11 @@
       <c r="F246" s="3" t="s">
         <v>1114</v>
       </c>
-      <c r="G246" s="2" t="s">
-        <v>134</v>
+      <c r="G246" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="H246" s="2" t="s">
-        <v>110</v>
+        <v>15</v>
       </c>
       <c r="I246" s="2" t="s">
         <v>16</v>
@@ -16272,30 +16263,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="247" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="247" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="2" t="n">
-        <v>246</v>
-      </c>
-      <c r="B247" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B247" s="4" t="s">
         <v>1115</v>
       </c>
-      <c r="C247" s="3" t="s">
+      <c r="C247" s="2" t="s">
         <v>1116</v>
       </c>
-      <c r="D247" s="3" t="s">
+      <c r="D247" s="2" t="s">
         <v>1117</v>
       </c>
-      <c r="E247" s="3" t="s">
+      <c r="E247" s="2" t="s">
         <v>1118</v>
       </c>
-      <c r="F247" s="3" t="s">
+      <c r="F247" s="2" t="s">
         <v>1119</v>
       </c>
       <c r="G247" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H247" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I247" s="2" t="s">
         <v>16</v>
@@ -16304,27 +16295,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="248" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="248" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="2" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B248" s="4" t="s">
         <v>1120</v>
       </c>
-      <c r="C248" s="2" t="s">
+      <c r="C248" s="3" t="s">
         <v>1121</v>
       </c>
-      <c r="D248" s="2" t="s">
+      <c r="D248" s="3" t="s">
         <v>1122</v>
       </c>
-      <c r="E248" s="2" t="s">
+      <c r="E248" s="3" t="s">
         <v>1123</v>
       </c>
-      <c r="F248" s="2" t="s">
+      <c r="F248" s="3" t="s">
         <v>1124</v>
       </c>
       <c r="G248" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H248" s="2" t="s">
         <v>38</v>
@@ -16336,30 +16327,32 @@
         <v>4</v>
       </c>
     </row>
-    <row r="249" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="249" customFormat="false" ht="50.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="2" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B249" s="4" t="s">
         <v>1125</v>
       </c>
-      <c r="C249" s="3" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D249" s="3" t="s">
-        <v>1127</v>
-      </c>
-      <c r="E249" s="3" t="s">
-        <v>1128</v>
-      </c>
-      <c r="F249" s="3" t="s">
-        <v>1129</v>
+      <c r="C249" s="3" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D249" s="3" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E249" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F249" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="G249" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H249" s="2" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="I249" s="2" t="s">
         <v>16</v>
@@ -16368,32 +16361,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="250" customFormat="false" ht="50.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="250" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="2" t="n">
-        <v>249</v>
-      </c>
-      <c r="B250" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="B250" s="2" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C250" s="2" t="s">
+        <v>1127</v>
+      </c>
+      <c r="D250" s="2" t="s">
+        <v>1128</v>
+      </c>
+      <c r="E250" s="2" t="s">
+        <v>1129</v>
+      </c>
+      <c r="F250" s="2" t="s">
         <v>1130</v>
       </c>
-      <c r="C250" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D250" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="E250" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F250" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="G250" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H250" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I250" s="2" t="s">
         <v>16</v>
@@ -16402,11 +16393,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="251" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="251" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="2" t="n">
-        <v>250</v>
-      </c>
-      <c r="B251" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B251" s="4" t="s">
         <v>1131</v>
       </c>
       <c r="C251" s="2" t="s">
@@ -16422,7 +16413,7 @@
         <v>1135</v>
       </c>
       <c r="G251" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H251" s="2" t="s">
         <v>38</v>
@@ -16434,11 +16425,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="252" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="252" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="2" t="n">
-        <v>251</v>
-      </c>
-      <c r="B252" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B252" s="2" t="s">
         <v>1136</v>
       </c>
       <c r="C252" s="2" t="s">
@@ -16454,7 +16445,7 @@
         <v>1140</v>
       </c>
       <c r="G252" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H252" s="2" t="s">
         <v>38</v>
@@ -16466,30 +16457,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="253" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="253" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="2" t="n">
-        <v>252</v>
-      </c>
-      <c r="B253" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B253" s="4" t="s">
         <v>1141</v>
       </c>
-      <c r="C253" s="2" t="s">
+      <c r="C253" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="D253" s="3" t="s">
         <v>1142</v>
       </c>
-      <c r="D253" s="2" t="s">
+      <c r="E253" s="2" t="s">
+        <v>850</v>
+      </c>
+      <c r="F253" s="3" t="s">
         <v>1143</v>
       </c>
-      <c r="E253" s="2" t="s">
-        <v>1144</v>
-      </c>
-      <c r="F253" s="2" t="s">
-        <v>1145</v>
-      </c>
       <c r="G253" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H253" s="2" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="I253" s="2" t="s">
         <v>16</v>
@@ -16498,30 +16489,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="254" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="254" customFormat="false" ht="88.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="2" t="n">
-        <v>253</v>
-      </c>
-      <c r="B254" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="B254" s="3" t="s">
+        <v>1144</v>
+      </c>
+      <c r="C254" s="2" t="s">
+        <v>1145</v>
+      </c>
+      <c r="D254" s="2" t="s">
         <v>1146</v>
       </c>
-      <c r="C254" s="3" t="n">
-        <v>123</v>
-      </c>
-      <c r="D254" s="3" t="s">
+      <c r="E254" s="2" t="s">
         <v>1147</v>
       </c>
-      <c r="E254" s="2" t="s">
-        <v>850</v>
-      </c>
-      <c r="F254" s="3" t="s">
+      <c r="F254" s="2" t="s">
         <v>1148</v>
       </c>
       <c r="G254" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H254" s="2" t="s">
-        <v>15</v>
+        <v>110</v>
       </c>
       <c r="I254" s="2" t="s">
         <v>16</v>
@@ -16530,24 +16521,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="255" customFormat="false" ht="88.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="255" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="2" t="n">
-        <v>254</v>
-      </c>
-      <c r="B255" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B255" s="4" t="s">
         <v>1149</v>
       </c>
-      <c r="C255" s="2" t="s">
+      <c r="C255" s="3" t="s">
         <v>1150</v>
       </c>
-      <c r="D255" s="2" t="s">
+      <c r="D255" s="3" t="s">
         <v>1151</v>
       </c>
-      <c r="E255" s="2" t="s">
+      <c r="E255" s="3" t="s">
         <v>1152</v>
       </c>
       <c r="F255" s="2" t="s">
-        <v>1153</v>
+        <v>638</v>
       </c>
       <c r="G255" s="2" t="n">
         <v>2</v>
@@ -16562,27 +16553,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="256" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="256" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="2" t="n">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B256" s="4" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C256" s="2" t="s">
         <v>1154</v>
       </c>
-      <c r="C256" s="3" t="s">
+      <c r="D256" s="2" t="s">
         <v>1155</v>
       </c>
-      <c r="D256" s="3" t="s">
+      <c r="E256" s="2" t="s">
         <v>1156</v>
       </c>
-      <c r="E256" s="3" t="s">
+      <c r="F256" s="3" t="s">
         <v>1157</v>
       </c>
-      <c r="F256" s="2" t="s">
-        <v>638</v>
-      </c>
       <c r="G256" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H256" s="2" t="s">
         <v>110</v>
@@ -16594,30 +16585,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="257" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="257" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="2" t="n">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B257" s="4" t="s">
         <v>1158</v>
       </c>
-      <c r="C257" s="2" t="s">
+      <c r="C257" s="3" t="s">
         <v>1159</v>
       </c>
-      <c r="D257" s="2" t="s">
+      <c r="D257" s="3" t="s">
         <v>1160</v>
       </c>
-      <c r="E257" s="2" t="s">
+      <c r="E257" s="3" t="s">
         <v>1161</v>
       </c>
       <c r="F257" s="3" t="s">
         <v>1162</v>
       </c>
       <c r="G257" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H257" s="2" t="s">
-        <v>110</v>
+        <v>38</v>
       </c>
       <c r="I257" s="2" t="s">
         <v>16</v>
@@ -16626,30 +16617,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="258" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="258" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="2" t="n">
-        <v>257</v>
-      </c>
-      <c r="B258" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B258" s="2" t="s">
         <v>1163</v>
       </c>
-      <c r="C258" s="3" t="s">
+      <c r="C258" s="2" t="s">
         <v>1164</v>
       </c>
-      <c r="D258" s="3" t="s">
+      <c r="D258" s="2" t="s">
         <v>1165</v>
       </c>
-      <c r="E258" s="3" t="s">
+      <c r="E258" s="2" t="s">
         <v>1166</v>
       </c>
-      <c r="F258" s="3" t="s">
+      <c r="F258" s="2" t="s">
         <v>1167</v>
       </c>
       <c r="G258" s="2" t="n">
         <v>3</v>
       </c>
       <c r="H258" s="2" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="I258" s="2" t="s">
         <v>16</v>
@@ -16658,30 +16649,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="259" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="259" customFormat="false" ht="50.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="2" t="n">
-        <v>258</v>
-      </c>
-      <c r="B259" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B259" s="4" t="s">
         <v>1168</v>
       </c>
-      <c r="C259" s="2" t="s">
+      <c r="C259" s="3" t="s">
+        <v>847</v>
+      </c>
+      <c r="D259" s="3" t="s">
         <v>1169</v>
       </c>
-      <c r="D259" s="2" t="s">
+      <c r="E259" s="3" t="s">
         <v>1170</v>
       </c>
-      <c r="E259" s="2" t="s">
+      <c r="F259" s="3" t="s">
         <v>1171</v>
-      </c>
-      <c r="F259" s="2" t="s">
-        <v>1172</v>
       </c>
       <c r="G259" s="2" t="n">
         <v>3</v>
       </c>
       <c r="H259" s="2" t="s">
-        <v>110</v>
+        <v>15</v>
       </c>
       <c r="I259" s="2" t="s">
         <v>16</v>
@@ -16690,30 +16681,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="260" customFormat="false" ht="50.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="260" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="2" t="n">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B260" s="4" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C260" s="3" t="s">
         <v>1173</v>
-      </c>
-      <c r="C260" s="3" t="s">
-        <v>847</v>
       </c>
       <c r="D260" s="3" t="s">
         <v>1174</v>
       </c>
       <c r="E260" s="3" t="s">
-        <v>1106</v>
+        <v>1175</v>
       </c>
       <c r="F260" s="3" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="G260" s="2" t="n">
         <v>3</v>
       </c>
       <c r="H260" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I260" s="2" t="s">
         <v>16</v>
@@ -16722,27 +16713,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="261" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="261" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="2" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B261" s="4" t="s">
-        <v>1176</v>
-      </c>
-      <c r="C261" s="3" t="s">
         <v>1177</v>
       </c>
-      <c r="D261" s="3" t="s">
+      <c r="C261" s="2" t="s">
         <v>1178</v>
       </c>
-      <c r="E261" s="3" t="s">
+      <c r="D261" s="2" t="s">
         <v>1179</v>
       </c>
-      <c r="F261" s="3" t="s">
+      <c r="E261" s="2" t="s">
         <v>1180</v>
       </c>
+      <c r="F261" s="2" t="s">
+        <v>1181</v>
+      </c>
       <c r="G261" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H261" s="2" t="s">
         <v>38</v>
@@ -16756,28 +16747,28 @@
     </row>
     <row r="262" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="2" t="n">
-        <v>261</v>
-      </c>
-      <c r="B262" s="4" t="s">
-        <v>1181</v>
-      </c>
-      <c r="C262" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B262" s="2" t="s">
         <v>1182</v>
       </c>
-      <c r="D262" s="2" t="s">
+      <c r="C262" s="3" t="s">
         <v>1183</v>
       </c>
-      <c r="E262" s="2" t="s">
+      <c r="D262" s="3" t="s">
         <v>1184</v>
       </c>
-      <c r="F262" s="2" t="s">
+      <c r="E262" s="3" t="s">
         <v>1185</v>
       </c>
+      <c r="F262" s="3" t="s">
+        <v>1186</v>
+      </c>
       <c r="G262" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H262" s="2" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="I262" s="2" t="s">
         <v>16</v>
@@ -16786,30 +16777,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="263" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="263" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="2" t="n">
-        <v>262</v>
-      </c>
-      <c r="B263" s="2" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C263" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B263" s="4" t="s">
         <v>1187</v>
       </c>
-      <c r="D263" s="3" t="s">
+      <c r="C263" s="2" t="s">
         <v>1188</v>
       </c>
-      <c r="E263" s="3" t="s">
+      <c r="D263" s="2" t="s">
         <v>1189</v>
       </c>
-      <c r="F263" s="3" t="s">
+      <c r="E263" s="2" t="s">
         <v>1190</v>
+      </c>
+      <c r="F263" s="2" t="s">
+        <v>1191</v>
       </c>
       <c r="G263" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H263" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I263" s="2" t="s">
         <v>16</v>
@@ -16818,27 +16809,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="264" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="264" customFormat="false" ht="97" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="2" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B264" s="4" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="D264" s="2" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="E264" s="2" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="F264" s="2" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="G264" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H264" s="2" t="s">
         <v>38</v>
@@ -16850,27 +16841,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="265" customFormat="false" ht="97" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="265" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="2" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B265" s="4" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="D265" s="2" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="E265" s="2" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="F265" s="2" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="G265" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H265" s="2" t="s">
         <v>38</v>
@@ -16882,30 +16873,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="266" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="266" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="2" t="n">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B266" s="4" t="s">
-        <v>1201</v>
-      </c>
-      <c r="C266" s="2" t="s">
         <v>1202</v>
       </c>
-      <c r="D266" s="2" t="s">
+      <c r="C266" s="4" t="s">
         <v>1203</v>
       </c>
-      <c r="E266" s="2" t="s">
+      <c r="D266" s="4" t="s">
         <v>1204</v>
       </c>
-      <c r="F266" s="2" t="s">
+      <c r="E266" s="4" t="s">
         <v>1205</v>
       </c>
+      <c r="F266" s="4" t="s">
+        <v>1206</v>
+      </c>
       <c r="G266" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H266" s="2" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="I266" s="2" t="s">
         <v>16</v>
@@ -16914,30 +16905,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="267" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="267" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="2" t="n">
-        <v>266</v>
-      </c>
-      <c r="B267" s="4" t="s">
-        <v>1206</v>
-      </c>
-      <c r="C267" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B267" s="2" t="s">
         <v>1207</v>
       </c>
-      <c r="D267" s="4" t="s">
+      <c r="C267" s="2" t="s">
         <v>1208</v>
       </c>
-      <c r="E267" s="4" t="s">
+      <c r="D267" s="2" t="s">
+        <v>998</v>
+      </c>
+      <c r="E267" s="2" t="s">
         <v>1209</v>
       </c>
-      <c r="F267" s="4" t="s">
+      <c r="F267" s="2" t="s">
         <v>1210</v>
       </c>
       <c r="G267" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H267" s="2" t="s">
-        <v>110</v>
+        <v>15</v>
       </c>
       <c r="I267" s="2" t="s">
         <v>16</v>
@@ -16946,30 +16937,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="268" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="268" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="2" t="n">
-        <v>267</v>
-      </c>
-      <c r="B268" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B268" s="4" t="s">
         <v>1211</v>
       </c>
-      <c r="C268" s="2" t="s">
+      <c r="C268" s="3" t="s">
         <v>1212</v>
       </c>
-      <c r="D268" s="2" t="s">
-        <v>998</v>
-      </c>
-      <c r="E268" s="2" t="s">
+      <c r="D268" s="3" t="s">
         <v>1213</v>
       </c>
-      <c r="F268" s="2" t="s">
+      <c r="E268" s="3" t="s">
         <v>1214</v>
       </c>
+      <c r="F268" s="3" t="s">
+        <v>1215</v>
+      </c>
       <c r="G268" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H268" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I268" s="2" t="s">
         <v>16</v>
@@ -16978,30 +16969,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="269" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="269" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="2" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B269" s="4" t="s">
-        <v>1215</v>
-      </c>
-      <c r="C269" s="3" t="s">
         <v>1216</v>
       </c>
-      <c r="D269" s="3" t="s">
+      <c r="C269" s="2" t="s">
         <v>1217</v>
       </c>
-      <c r="E269" s="3" t="s">
+      <c r="D269" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="F269" s="3" t="s">
+      <c r="E269" s="2" t="s">
         <v>1219</v>
       </c>
+      <c r="F269" s="2" t="s">
+        <v>1220</v>
+      </c>
       <c r="G269" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H269" s="2" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="I269" s="2" t="s">
         <v>16</v>
@@ -17010,30 +17001,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="270" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="270" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A270" s="2" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B270" s="4" t="s">
-        <v>1220</v>
-      </c>
-      <c r="C270" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="D270" s="2" t="s">
+      <c r="C270" s="3" t="s">
         <v>1222</v>
       </c>
-      <c r="E270" s="2" t="s">
+      <c r="D270" s="3" t="s">
         <v>1223</v>
       </c>
+      <c r="E270" s="3" t="s">
+        <v>1224</v>
+      </c>
       <c r="F270" s="2" t="s">
-        <v>1224</v>
+        <v>850</v>
       </c>
       <c r="G270" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H270" s="2" t="s">
-        <v>110</v>
+        <v>38</v>
       </c>
       <c r="I270" s="2" t="s">
         <v>16</v>
@@ -17042,9 +17033,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="271" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="271" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="2" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B271" s="4" t="s">
         <v>1225</v>
@@ -17058,14 +17049,14 @@
       <c r="E271" s="3" t="s">
         <v>1228</v>
       </c>
-      <c r="F271" s="2" t="s">
-        <v>850</v>
+      <c r="F271" s="3" t="s">
+        <v>1229</v>
       </c>
       <c r="G271" s="2" t="n">
         <v>3</v>
       </c>
       <c r="H271" s="2" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="I271" s="2" t="s">
         <v>16</v>
@@ -17074,27 +17065,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="272" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="272" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="2" t="n">
-        <v>271</v>
-      </c>
-      <c r="B272" s="4" t="s">
-        <v>1229</v>
-      </c>
-      <c r="C272" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="B272" s="2" t="s">
         <v>1230</v>
       </c>
-      <c r="D272" s="3" t="s">
+      <c r="C272" s="2" t="s">
         <v>1231</v>
       </c>
-      <c r="E272" s="3" t="s">
+      <c r="D272" s="2" t="s">
         <v>1232</v>
       </c>
-      <c r="F272" s="3" t="s">
+      <c r="E272" s="2" t="s">
         <v>1233</v>
       </c>
+      <c r="F272" s="2" t="s">
+        <v>1234</v>
+      </c>
       <c r="G272" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H272" s="2" t="s">
         <v>15</v>
@@ -17106,30 +17097,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="273" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="273" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="2" t="n">
-        <v>272</v>
-      </c>
-      <c r="B273" s="2" t="s">
-        <v>1234</v>
-      </c>
-      <c r="C273" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="B273" s="4" t="s">
         <v>1235</v>
       </c>
+      <c r="C273" s="3" t="s">
+        <v>1236</v>
+      </c>
       <c r="D273" s="2" t="s">
-        <v>1236</v>
-      </c>
-      <c r="E273" s="2" t="s">
+        <v>850</v>
+      </c>
+      <c r="E273" s="3" t="s">
         <v>1237</v>
       </c>
-      <c r="F273" s="2" t="s">
+      <c r="F273" s="3" t="s">
         <v>1238</v>
       </c>
       <c r="G273" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H273" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I273" s="2" t="s">
         <v>16</v>
@@ -17138,27 +17129,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="274" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="274" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="2" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B274" s="4" t="s">
         <v>1239</v>
       </c>
-      <c r="C274" s="3" t="s">
+      <c r="C274" s="2" t="s">
         <v>1240</v>
       </c>
-      <c r="D274" s="2" t="s">
-        <v>850</v>
-      </c>
-      <c r="E274" s="3" t="s">
+      <c r="D274" s="4" t="s">
         <v>1241</v>
       </c>
-      <c r="F274" s="3" t="s">
+      <c r="E274" s="2" t="s">
         <v>1242</v>
       </c>
+      <c r="F274" s="2" t="s">
+        <v>1243</v>
+      </c>
       <c r="G274" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H274" s="2" t="s">
         <v>38</v>
@@ -17170,27 +17161,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="275" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="275" customFormat="false" ht="88.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="2" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B275" s="4" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>1244</v>
-      </c>
-      <c r="D275" s="4" t="s">
         <v>1245</v>
       </c>
+      <c r="D275" s="2" t="s">
+        <v>1246</v>
+      </c>
       <c r="E275" s="2" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="F275" s="2" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="G275" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H275" s="2" t="s">
         <v>38</v>
@@ -17202,24 +17193,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="276" customFormat="false" ht="88.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="276" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="2" t="n">
-        <v>275</v>
-      </c>
-      <c r="B276" s="4" t="s">
-        <v>1248</v>
+        <v>276</v>
+      </c>
+      <c r="B276" s="2" t="s">
+        <v>1249</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="D276" s="2" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="E276" s="2" t="s">
-        <v>1251</v>
-      </c>
-      <c r="F276" s="2" t="s">
         <v>1252</v>
+      </c>
+      <c r="F276" s="4" t="s">
+        <v>1253</v>
       </c>
       <c r="G276" s="2" t="n">
         <v>3</v>
@@ -17234,30 +17225,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="277" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="277" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="2" t="n">
-        <v>276</v>
-      </c>
-      <c r="B277" s="2" t="s">
-        <v>1253</v>
-      </c>
-      <c r="C277" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B277" s="4" t="s">
         <v>1254</v>
       </c>
-      <c r="D277" s="2" t="s">
+      <c r="C277" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D277" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E277" s="3" t="s">
         <v>1255</v>
       </c>
-      <c r="E277" s="2" t="s">
+      <c r="F277" s="3" t="s">
         <v>1256</v>
       </c>
-      <c r="F277" s="4" t="s">
-        <v>1257</v>
-      </c>
       <c r="G277" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H277" s="2" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="I277" s="2" t="s">
         <v>16</v>
@@ -17266,30 +17257,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="278" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="278" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="2" t="n">
-        <v>277</v>
-      </c>
-      <c r="B278" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B278" s="2" t="s">
+        <v>1257</v>
+      </c>
+      <c r="C278" s="2" t="s">
         <v>1258</v>
       </c>
-      <c r="C278" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D278" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E278" s="3" t="s">
+      <c r="D278" s="2" t="s">
         <v>1259</v>
       </c>
-      <c r="F278" s="3" t="s">
+      <c r="E278" s="2" t="s">
         <v>1260</v>
       </c>
+      <c r="F278" s="2" t="s">
+        <v>1261</v>
+      </c>
       <c r="G278" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H278" s="2" t="s">
-        <v>110</v>
+        <v>38</v>
       </c>
       <c r="I278" s="2" t="s">
         <v>16</v>
@@ -17300,28 +17291,28 @@
     </row>
     <row r="279" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="2" t="n">
-        <v>278</v>
-      </c>
-      <c r="B279" s="2" t="s">
-        <v>1261</v>
+        <v>279</v>
+      </c>
+      <c r="B279" s="4" t="s">
+        <v>1262</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="D279" s="2" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="E279" s="2" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="F279" s="2" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="G279" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H279" s="2" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="I279" s="2" t="s">
         <v>16</v>
@@ -17330,27 +17321,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="280" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="280" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="2" t="n">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B280" s="4" t="s">
-        <v>1266</v>
-      </c>
-      <c r="C280" s="2" t="s">
         <v>1267</v>
       </c>
-      <c r="D280" s="2" t="s">
+      <c r="C280" s="3" t="s">
         <v>1268</v>
       </c>
-      <c r="E280" s="2" t="s">
+      <c r="D280" s="3" t="s">
         <v>1269</v>
       </c>
-      <c r="F280" s="2" t="s">
+      <c r="E280" s="3" t="s">
         <v>1270</v>
       </c>
-      <c r="G280" s="2" t="n">
-        <v>3</v>
+      <c r="F280" s="3" t="s">
+        <v>1271</v>
+      </c>
+      <c r="G280" s="2" t="s">
+        <v>1272</v>
       </c>
       <c r="H280" s="2" t="s">
         <v>110</v>
@@ -17362,47 +17353,47 @@
         <v>4</v>
       </c>
     </row>
-    <row r="281" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="281" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="2" t="n">
-        <v>280</v>
-      </c>
-      <c r="B281" s="4" t="s">
-        <v>1271</v>
-      </c>
-      <c r="C281" s="3" t="s">
-        <v>1272</v>
-      </c>
-      <c r="D281" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B281" s="2" t="s">
         <v>1273</v>
       </c>
-      <c r="E281" s="3" t="s">
+      <c r="C281" s="2" t="s">
         <v>1274</v>
       </c>
-      <c r="F281" s="3" t="s">
+      <c r="D281" s="2" t="s">
         <v>1275</v>
       </c>
-      <c r="G281" s="2" t="s">
+      <c r="E281" s="2" t="s">
         <v>1276</v>
       </c>
+      <c r="F281" s="2" t="s">
+        <v>1277</v>
+      </c>
+      <c r="G281" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="H281" s="2" t="s">
-        <v>110</v>
+        <v>15</v>
       </c>
       <c r="I281" s="2" t="s">
         <v>16</v>
       </c>
       <c r="J281" s="2" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="282" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="282" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="2" t="n">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>1278</v>
+        <v>384</v>
       </c>
       <c r="D282" s="2" t="s">
         <v>1279</v>
@@ -17426,30 +17417,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="215.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="2" t="n">
-        <v>282</v>
-      </c>
-      <c r="B283" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B283" s="4" t="s">
         <v>1282</v>
       </c>
-      <c r="C283" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="D283" s="2" t="s">
+      <c r="C283" s="3" t="s">
         <v>1283</v>
       </c>
-      <c r="E283" s="2" t="s">
+      <c r="D283" s="3" t="s">
         <v>1284</v>
       </c>
-      <c r="F283" s="2" t="s">
+      <c r="E283" s="3" t="s">
         <v>1285</v>
       </c>
+      <c r="F283" s="3" t="s">
+        <v>1286</v>
+      </c>
       <c r="G283" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H283" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I283" s="2" t="s">
         <v>16</v>
@@ -17458,27 +17449,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="284" customFormat="false" ht="215.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="284" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="2" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B284" s="4" t="s">
-        <v>1286</v>
-      </c>
-      <c r="C284" s="3" t="s">
         <v>1287</v>
       </c>
-      <c r="D284" s="3" t="s">
+      <c r="C284" s="2" t="s">
         <v>1288</v>
       </c>
-      <c r="E284" s="3" t="s">
+      <c r="D284" s="2" t="s">
         <v>1289</v>
       </c>
-      <c r="F284" s="3" t="s">
+      <c r="E284" s="2" t="s">
         <v>1290</v>
       </c>
+      <c r="F284" s="2" t="s">
+        <v>1291</v>
+      </c>
       <c r="G284" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H284" s="2" t="s">
         <v>38</v>
@@ -17490,24 +17481,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="285" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="285" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="2" t="n">
-        <v>284</v>
-      </c>
-      <c r="B285" s="4" t="s">
-        <v>1291</v>
+        <v>285</v>
+      </c>
+      <c r="B285" s="2" t="s">
+        <v>1292</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="D285" s="2" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="E285" s="2" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="F285" s="2" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
       <c r="G285" s="2" t="n">
         <v>2</v>
@@ -17522,30 +17513,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="286" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="286" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="2" t="n">
-        <v>285</v>
-      </c>
-      <c r="B286" s="2" t="s">
-        <v>1296</v>
-      </c>
-      <c r="C286" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B286" s="4" t="s">
         <v>1297</v>
       </c>
-      <c r="D286" s="2" t="s">
+      <c r="C286" s="3" t="s">
         <v>1298</v>
       </c>
-      <c r="E286" s="2" t="s">
+      <c r="D286" s="3" t="s">
         <v>1299</v>
       </c>
-      <c r="F286" s="2" t="s">
+      <c r="E286" s="3" t="s">
         <v>1300</v>
       </c>
+      <c r="F286" s="3" t="s">
+        <v>1301</v>
+      </c>
       <c r="G286" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H286" s="2" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="I286" s="2" t="s">
         <v>16</v>
@@ -17554,30 +17545,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="287" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="287" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="2" t="n">
-        <v>286</v>
-      </c>
-      <c r="B287" s="4" t="s">
-        <v>1301</v>
+        <v>287</v>
+      </c>
+      <c r="B287" s="2" t="s">
+        <v>1302</v>
       </c>
       <c r="C287" s="3" t="s">
-        <v>1302</v>
+        <v>1303</v>
       </c>
       <c r="D287" s="3" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="E287" s="3" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="F287" s="3" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="G287" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H287" s="2" t="s">
-        <v>15</v>
+        <v>110</v>
       </c>
       <c r="I287" s="2" t="s">
         <v>16</v>
@@ -17588,28 +17579,28 @@
     </row>
     <row r="288" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="2" t="n">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>1306</v>
-      </c>
-      <c r="C288" s="3" t="s">
         <v>1307</v>
       </c>
-      <c r="D288" s="3" t="s">
+      <c r="C288" s="2" t="s">
         <v>1308</v>
       </c>
-      <c r="E288" s="3" t="s">
+      <c r="D288" s="2" t="s">
         <v>1309</v>
       </c>
-      <c r="F288" s="3" t="s">
+      <c r="E288" s="2" t="s">
         <v>1310</v>
       </c>
+      <c r="F288" s="2" t="s">
+        <v>1311</v>
+      </c>
       <c r="G288" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H288" s="2" t="s">
-        <v>110</v>
+        <v>15</v>
       </c>
       <c r="I288" s="2" t="s">
         <v>16</v>
@@ -17618,30 +17609,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="289" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="289" customFormat="false" ht="139.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="2" t="n">
-        <v>288</v>
-      </c>
-      <c r="B289" s="2" t="s">
-        <v>1311</v>
+        <v>289</v>
+      </c>
+      <c r="B289" s="4" t="s">
+        <v>1312</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="D289" s="2" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="E289" s="2" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="F289" s="2" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="G289" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H289" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I289" s="2" t="s">
         <v>16</v>
@@ -17650,24 +17641,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="290" customFormat="false" ht="139.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="290" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="2" t="n">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B290" s="4" t="s">
-        <v>1316</v>
-      </c>
-      <c r="C290" s="2" t="s">
         <v>1317</v>
       </c>
-      <c r="D290" s="2" t="s">
+      <c r="C290" s="3" t="s">
         <v>1318</v>
       </c>
-      <c r="E290" s="2" t="s">
+      <c r="D290" s="3" t="s">
         <v>1319</v>
       </c>
-      <c r="F290" s="2" t="s">
+      <c r="E290" s="3" t="s">
         <v>1320</v>
+      </c>
+      <c r="F290" s="3" t="s">
+        <v>1321</v>
       </c>
       <c r="G290" s="2" t="n">
         <v>2</v>
@@ -17682,30 +17673,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="291" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="291" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="2" t="n">
-        <v>290</v>
-      </c>
-      <c r="B291" s="4" t="s">
-        <v>1321</v>
-      </c>
-      <c r="C291" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="B291" s="2" t="s">
         <v>1322</v>
       </c>
-      <c r="D291" s="3" t="s">
+      <c r="C291" s="2" t="s">
         <v>1323</v>
       </c>
-      <c r="E291" s="3" t="s">
+      <c r="D291" s="2" t="s">
         <v>1324</v>
       </c>
-      <c r="F291" s="3" t="s">
+      <c r="E291" s="2" t="s">
         <v>1325</v>
       </c>
+      <c r="F291" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="G291" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H291" s="2" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="I291" s="2" t="s">
         <v>16</v>
@@ -17714,30 +17705,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="292" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="292" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="2" t="n">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="D292" s="2" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="E292" s="2" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="F292" s="2" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="G292" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H292" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I292" s="2" t="s">
         <v>16</v>
@@ -17746,30 +17737,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="293" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="293" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="2" t="n">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="D293" s="2" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="E293" s="2" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="F293" s="2" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="G293" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H293" s="2" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="I293" s="2" t="s">
         <v>16</v>
@@ -17778,30 +17769,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="294" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="294" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A294" s="2" t="n">
-        <v>293</v>
-      </c>
-      <c r="B294" s="2" t="s">
-        <v>1336</v>
-      </c>
-      <c r="C294" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B294" s="4" t="s">
         <v>1337</v>
       </c>
-      <c r="D294" s="2" t="s">
+      <c r="C294" s="3" t="s">
         <v>1338</v>
       </c>
-      <c r="E294" s="2" t="s">
+      <c r="D294" s="3" t="s">
         <v>1339</v>
       </c>
-      <c r="F294" s="2" t="s">
+      <c r="E294" s="3" t="s">
         <v>1340</v>
       </c>
+      <c r="F294" s="3" t="s">
+        <v>1341</v>
+      </c>
       <c r="G294" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H294" s="2" t="s">
-        <v>110</v>
+        <v>38</v>
       </c>
       <c r="I294" s="2" t="s">
         <v>16</v>
@@ -17810,30 +17801,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="295" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="295" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A295" s="2" t="n">
-        <v>294</v>
-      </c>
-      <c r="B295" s="4" t="s">
-        <v>1341</v>
-      </c>
-      <c r="C295" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="B295" s="2" t="s">
         <v>1342</v>
       </c>
-      <c r="D295" s="3" t="s">
+      <c r="C295" s="2" t="s">
         <v>1343</v>
       </c>
-      <c r="E295" s="3" t="s">
+      <c r="D295" s="2" t="s">
         <v>1344</v>
       </c>
-      <c r="F295" s="3" t="s">
+      <c r="E295" s="2" t="s">
         <v>1345</v>
       </c>
+      <c r="F295" s="2" t="s">
+        <v>643</v>
+      </c>
       <c r="G295" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H295" s="2" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="I295" s="2" t="s">
         <v>16</v>
@@ -17842,30 +17833,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="296" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="296" customFormat="false" ht="255.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="2" t="n">
-        <v>295</v>
-      </c>
-      <c r="B296" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B296" s="4" t="s">
         <v>1346</v>
       </c>
-      <c r="C296" s="2" t="s">
+      <c r="C296" s="3" t="s">
         <v>1347</v>
       </c>
-      <c r="D296" s="2" t="s">
+      <c r="D296" s="3" t="s">
         <v>1348</v>
       </c>
-      <c r="E296" s="2" t="s">
+      <c r="E296" s="3" t="s">
         <v>1349</v>
       </c>
-      <c r="F296" s="2" t="s">
-        <v>643</v>
+      <c r="F296" s="3" t="s">
+        <v>1350</v>
       </c>
       <c r="G296" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H296" s="2" t="s">
-        <v>15</v>
+        <v>110</v>
       </c>
       <c r="I296" s="2" t="s">
         <v>16</v>
@@ -17874,30 +17865,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="297" customFormat="false" ht="255.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="297" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A297" s="2" t="n">
-        <v>296</v>
-      </c>
-      <c r="B297" s="4" t="s">
-        <v>1350</v>
-      </c>
-      <c r="C297" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="B297" s="2" t="s">
         <v>1351</v>
       </c>
-      <c r="D297" s="3" t="s">
+      <c r="C297" s="2" t="s">
         <v>1352</v>
       </c>
-      <c r="E297" s="3" t="s">
+      <c r="D297" s="2" t="s">
         <v>1353</v>
       </c>
-      <c r="F297" s="3" t="s">
+      <c r="E297" s="2" t="s">
         <v>1354</v>
       </c>
+      <c r="F297" s="2" t="s">
+        <v>1355</v>
+      </c>
       <c r="G297" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H297" s="2" t="s">
-        <v>110</v>
+        <v>38</v>
       </c>
       <c r="I297" s="2" t="s">
         <v>16</v>
@@ -17906,27 +17897,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="298" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="298" customFormat="false" ht="267.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="2" t="n">
-        <v>297</v>
-      </c>
-      <c r="B298" s="2" t="s">
-        <v>1355</v>
-      </c>
-      <c r="C298" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B298" s="4" t="s">
         <v>1356</v>
       </c>
-      <c r="D298" s="2" t="s">
+      <c r="C298" s="3" t="s">
         <v>1357</v>
       </c>
-      <c r="E298" s="2" t="s">
+      <c r="D298" s="3" t="s">
         <v>1358</v>
       </c>
-      <c r="F298" s="2" t="s">
+      <c r="E298" s="3" t="s">
         <v>1359</v>
       </c>
+      <c r="F298" s="3" t="s">
+        <v>1360</v>
+      </c>
       <c r="G298" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H298" s="2" t="s">
         <v>38</v>
@@ -17938,27 +17929,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="299" customFormat="false" ht="267.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="299" customFormat="false" ht="133.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="2" t="n">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B299" s="4" t="s">
-        <v>1360</v>
-      </c>
-      <c r="C299" s="3" t="s">
         <v>1361</v>
       </c>
-      <c r="D299" s="3" t="s">
+      <c r="C299" s="2" t="s">
         <v>1362</v>
       </c>
-      <c r="E299" s="3" t="s">
+      <c r="D299" s="2" t="s">
         <v>1363</v>
       </c>
-      <c r="F299" s="3" t="s">
+      <c r="E299" s="2" t="s">
         <v>1364</v>
       </c>
+      <c r="F299" s="2" t="s">
+        <v>1365</v>
+      </c>
       <c r="G299" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H299" s="2" t="s">
         <v>38</v>
@@ -17970,67 +17961,35 @@
         <v>5</v>
       </c>
     </row>
-    <row r="300" customFormat="false" ht="133.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="300" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A300" s="2" t="n">
-        <v>299</v>
-      </c>
-      <c r="B300" s="4" t="s">
-        <v>1365</v>
-      </c>
-      <c r="C300" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B300" s="2" t="s">
         <v>1366</v>
       </c>
-      <c r="D300" s="2" t="s">
+      <c r="C300" s="4" t="s">
         <v>1367</v>
       </c>
-      <c r="E300" s="2" t="s">
+      <c r="D300" s="4" t="s">
         <v>1368</v>
       </c>
-      <c r="F300" s="2" t="s">
+      <c r="E300" s="4" t="s">
         <v>1369</v>
       </c>
+      <c r="F300" s="4" t="s">
+        <v>1370</v>
+      </c>
       <c r="G300" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H300" s="2" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="I300" s="2" t="s">
         <v>16</v>
       </c>
       <c r="J300" s="2" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="301" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A301" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="B301" s="2" t="s">
-        <v>1370</v>
-      </c>
-      <c r="C301" s="4" t="s">
-        <v>1371</v>
-      </c>
-      <c r="D301" s="4" t="s">
-        <v>1372</v>
-      </c>
-      <c r="E301" s="4" t="s">
-        <v>1373</v>
-      </c>
-      <c r="F301" s="4" t="s">
-        <v>1374</v>
-      </c>
-      <c r="G301" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H301" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I301" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J301" s="2" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>